<commit_message>
Re-enable ILMP with propoer upper bound initialization.
</commit_message>
<xml_diff>
--- a/data/rts_24_data.xlsx
+++ b/data/rts_24_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\repos\aro_tnep_sb_local\aro_tnep_sb\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D400EA6-313C-4264-BF07-2AFDDF50079B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F8119E0-502C-40D1-AC79-F81887BD335C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6345" yWindow="3825" windowWidth="28800" windowHeight="15345" firstSheet="1" activeTab="2" xr2:uid="{61A108C2-359E-4CFD-B8CB-B26F47640E97}"/>
   </bookViews>
@@ -22,17 +22,19 @@
     <sheet name="RES" sheetId="4" r:id="rId7"/>
     <sheet name="ESS" sheetId="2" r:id="rId8"/>
     <sheet name="ESS_can" sheetId="15" r:id="rId9"/>
-    <sheet name="loads" sheetId="5" r:id="rId10"/>
-    <sheet name="loads_static" sheetId="14" r:id="rId11"/>
-    <sheet name="UB" sheetId="11" r:id="rId12"/>
+    <sheet name="ESS_none" sheetId="17" r:id="rId10"/>
+    <sheet name="loads" sheetId="5" r:id="rId11"/>
+    <sheet name="loads_static" sheetId="14" r:id="rId12"/>
+    <sheet name="UB" sheetId="11" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="ExternalData_1" localSheetId="4" hidden="1">CG!$A$1:$I$11</definedName>
     <definedName name="ExternalData_1" localSheetId="5" hidden="1">CG_static!$A$1:$I$11</definedName>
     <definedName name="ExternalData_1" localSheetId="7" hidden="1">ESS!$A$1:$I$6</definedName>
     <definedName name="ExternalData_1" localSheetId="8" hidden="1">ESS_can!$A$1:$I$25</definedName>
-    <definedName name="ExternalData_1" localSheetId="9" hidden="1">loads!$A$1:$F$18</definedName>
-    <definedName name="ExternalData_1" localSheetId="10" hidden="1">loads_static!$A$1:$F$18</definedName>
+    <definedName name="ExternalData_1" localSheetId="9" hidden="1">ESS_none!$A$1:$I$25</definedName>
+    <definedName name="ExternalData_1" localSheetId="10" hidden="1">loads!$A$1:$F$18</definedName>
+    <definedName name="ExternalData_1" localSheetId="11" hidden="1">loads_static!$A$1:$F$18</definedName>
     <definedName name="ExternalData_1" localSheetId="6" hidden="1">RES!$A$1:$G$11</definedName>
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">TL!$A$2:$F$56</definedName>
     <definedName name="ExternalData_1" localSheetId="2" hidden="1">TL_ESS!$A$2:$F$73</definedName>
@@ -138,7 +140,15 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="9" xr16:uid="{48047EF9-8182-45BF-9406-6828FCB3C1DB}" name="Query - Table013 (Page 7)" description="Connection to the 'Table013 (Page 7)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="9" xr16:uid="{972F0B14-A797-4BB3-B12E-D9736EE801F3}" keepAlive="1" name="ModelConnection_ExternalData_18" description="Data Model" type="5" refreshedVersion="8" minRefreshableVersion="5" saveData="1">
+    <dbPr connection="Data Model Connection" command="Table015  Page 81" commandType="3"/>
+    <extLst>
+      <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
+        <x15:connection id="" model="1"/>
+      </ext>
+    </extLst>
+  </connection>
+  <connection id="10" xr16:uid="{48047EF9-8182-45BF-9406-6828FCB3C1DB}" name="Query - Table013 (Page 7)" description="Connection to the 'Table013 (Page 7)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="8c04846e-574b-49a9-b03c-b2747427d9dd">
@@ -151,7 +161,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="10" xr16:uid="{D25222F1-44AE-41FD-9C1A-34D8EC774F85}" name="Query - Table015 (Page 8)" description="Connection to the 'Table015 (Page 8)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="11" xr16:uid="{D25222F1-44AE-41FD-9C1A-34D8EC774F85}" name="Query - Table015 (Page 8)" description="Connection to the 'Table015 (Page 8)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="de4b364e-904d-453f-b309-9b29f4b6980b">
@@ -164,7 +174,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="11" xr16:uid="{9BE9130A-2930-4B7E-970E-BB06E9BF2541}" name="Query - Table015 (Page 8) (2)" description="Connection to the 'Table015 (Page 8) (2)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="12" xr16:uid="{9BE9130A-2930-4B7E-970E-BB06E9BF2541}" name="Query - Table015 (Page 8) (2)" description="Connection to the 'Table015 (Page 8) (2)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="bab8510e-8513-42ad-9cdf-1ac3ec4e9f1b">
@@ -177,7 +187,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="12" xr16:uid="{DB7B854D-31F1-4986-87EA-28D7E3F22A40}" name="Query - Table016 (Page 9)" description="Connection to the 'Table016 (Page 9)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="13" xr16:uid="{DB7B854D-31F1-4986-87EA-28D7E3F22A40}" name="Query - Table016 (Page 9)" description="Connection to the 'Table016 (Page 9)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="cac904aa-0e22-4628-a796-1353ff5a529d">
@@ -190,7 +200,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="13" xr16:uid="{59C9E23C-4A77-4FEB-8B7C-246516601062}" name="Query - Table017 (Page 10)" description="Connection to the 'Table017 (Page 10)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="14" xr16:uid="{59C9E23C-4A77-4FEB-8B7C-246516601062}" name="Query - Table017 (Page 10)" description="Connection to the 'Table017 (Page 10)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="d74bc432-1696-4381-8eaf-73d554f2c018">
@@ -203,7 +213,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="14" xr16:uid="{1721F4CF-7B60-4608-93AB-FAF0432B15AC}" name="Query - Table018 (Page 11)" description="Connection to the 'Table018 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="15" xr16:uid="{1721F4CF-7B60-4608-93AB-FAF0432B15AC}" name="Query - Table018 (Page 11)" description="Connection to the 'Table018 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="8c5efc9b-d372-436d-99c1-dde23be08897">
@@ -216,7 +226,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="15" xr16:uid="{A1A23163-EB73-4407-B25D-E8015E90F7B2}" name="Query - Table019 (Page 11)" description="Connection to the 'Table019 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="16" xr16:uid="{A1A23163-EB73-4407-B25D-E8015E90F7B2}" name="Query - Table019 (Page 11)" description="Connection to the 'Table019 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="4003258f-51d4-4a29-b633-006a99e36f39">
@@ -229,7 +239,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="16" xr16:uid="{36980317-2A15-439E-97F5-1B37DA855CA7}" name="Query - Table020 (Page 11)" description="Connection to the 'Table020 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="17" xr16:uid="{36980317-2A15-439E-97F5-1B37DA855CA7}" name="Query - Table020 (Page 11)" description="Connection to the 'Table020 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="1684410c-15f4-46ac-9515-2721589996c3">
@@ -242,7 +252,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="17" xr16:uid="{91658BA7-C2B7-40CF-85C1-B529B7691349}" keepAlive="1" name="ThisWorkbookDataModel" description="Data Model" type="5" refreshedVersion="8" minRefreshableVersion="5" background="1">
+  <connection id="18" xr16:uid="{91658BA7-C2B7-40CF-85C1-B529B7691349}" keepAlive="1" name="ThisWorkbookDataModel" description="Data Model" type="5" refreshedVersion="8" minRefreshableVersion="5" background="1">
     <dbPr connection="Data Model Connection" command="Model" commandType="1"/>
     <olapPr sendLocale="1" rowDrillCount="1000"/>
     <extLst>
@@ -255,7 +265,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="91">
   <si>
     <t>Bus</t>
   </si>
@@ -629,7 +639,37 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="44">
+  <dxfs count="54">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -925,6 +965,34 @@
 </file>
 
 <file path=xl/queryTables/queryTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" headers="0" backgroundRefresh="0" connectionId="9" xr16:uid="{4E7C1BC1-84F6-4B3D-9B97-4C4110DDC440}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
+  <queryTableRefresh headersInLastRefresh="0" nextId="13" unboundColumnsRight="2">
+    <queryTableFields count="11">
+      <queryTableField id="1" name="Column1" tableColumnId="1"/>
+      <queryTableField id="2" name="Column2" tableColumnId="2"/>
+      <queryTableField id="3" name="Column3" tableColumnId="3"/>
+      <queryTableField id="4" name="Column4" tableColumnId="4"/>
+      <queryTableField id="5" name="Column5" tableColumnId="5"/>
+      <queryTableField id="6" name="Column6" tableColumnId="6"/>
+      <queryTableField id="10" dataBound="0" tableColumnId="9"/>
+      <queryTableField id="7" name="Column7" tableColumnId="7"/>
+      <queryTableField id="8" name="Column8" tableColumnId="8"/>
+      <queryTableField id="11" dataBound="0" tableColumnId="10"/>
+      <queryTableField id="12" dataBound="0" tableColumnId="11"/>
+    </queryTableFields>
+    <queryTableDeletedFields count="1">
+      <deletedField name="Column9"/>
+    </queryTableDeletedFields>
+  </queryTableRefresh>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{883FBD77-0823-4a55-B5E3-86C4891E6966}">
+      <x15:queryTable sourceDataName="Query - Table015 (Page 8) (2)"/>
+    </ext>
+  </extLst>
+</queryTable>
+</file>
+
+<file path=xl/queryTables/queryTable7.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" headers="0" backgroundRefresh="0" connectionId="5" xr16:uid="{77BA2001-87C6-4EE8-8DEC-2CF48E447D8D}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh headersInLastRefresh="0" nextId="11" unboundColumnsRight="2">
     <queryTableFields count="8">
@@ -950,7 +1018,7 @@
 </queryTable>
 </file>
 
-<file path=xl/queryTables/queryTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/queryTables/queryTable8.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" headers="0" backgroundRefresh="0" connectionId="7" xr16:uid="{BBD31A0C-45D3-4FA2-866B-846728885DB5}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh headersInLastRefresh="0" nextId="11" unboundColumnsRight="2">
     <queryTableFields count="8">
@@ -979,19 +1047,19 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C87D8478-344A-496F-AAA6-8F569A7D4D40}" name="Table016__Page_9" displayName="Table016__Page_9" ref="A1:M11" tableType="queryTable" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{79D75305-4854-43BA-B2CB-A34DF52B399C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{348BFC5E-8C9D-4A28-AE26-7E36A24B29D5}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{A9C2F495-5A0E-436F-BDB6-949DB67AD98C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{79D75305-4854-43BA-B2CB-A34DF52B399C}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{348BFC5E-8C9D-4A28-AE26-7E36A24B29D5}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{A9C2F495-5A0E-436F-BDB6-949DB67AD98C}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="51"/>
     <tableColumn id="3" xr3:uid="{7FF774DB-0D67-40A9-B982-C52DA09DF792}" uniqueName="3" name="Column3" queryTableFieldId="10"/>
     <tableColumn id="13" xr3:uid="{38D9054A-4E1E-4C27-A2EB-BF1275C9C20F}" uniqueName="13" name="Column13" queryTableFieldId="16"/>
-    <tableColumn id="5" xr3:uid="{EC2BA75E-8217-4AB8-973A-5FE762BAA906}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{EC2BA75E-8217-4AB8-973A-5FE762BAA906}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="50"/>
     <tableColumn id="12" xr3:uid="{0EA5DF1D-7231-49CD-911C-16E3792CFB3C}" uniqueName="12" name="Column12" queryTableFieldId="15"/>
-    <tableColumn id="6" xr3:uid="{F55F917B-81DF-4EBA-AB86-F0BA405A4CF7}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{11C3A255-1226-4232-9BB6-78B67B19A56C}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="38"/>
-    <tableColumn id="8" xr3:uid="{2B8A00F7-31A2-4F6B-A608-FA94DC8A6224}" uniqueName="8" name="Column8" queryTableFieldId="11" dataDxfId="37"/>
-    <tableColumn id="9" xr3:uid="{D55306F8-7304-4D19-A281-8D519DC063E7}" uniqueName="9" name="Column9" queryTableFieldId="12" dataDxfId="36"/>
-    <tableColumn id="10" xr3:uid="{1A472152-C9E9-412C-9F83-DF03AF116761}" uniqueName="10" name="Column10" queryTableFieldId="13" dataDxfId="35"/>
-    <tableColumn id="11" xr3:uid="{56D2129F-0933-4401-95C4-4829FF923A13}" uniqueName="11" name="Column11" queryTableFieldId="14" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{F55F917B-81DF-4EBA-AB86-F0BA405A4CF7}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{11C3A255-1226-4232-9BB6-78B67B19A56C}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{2B8A00F7-31A2-4F6B-A608-FA94DC8A6224}" uniqueName="8" name="Column8" queryTableFieldId="11" dataDxfId="47"/>
+    <tableColumn id="9" xr3:uid="{D55306F8-7304-4D19-A281-8D519DC063E7}" uniqueName="9" name="Column9" queryTableFieldId="12" dataDxfId="46"/>
+    <tableColumn id="10" xr3:uid="{1A472152-C9E9-412C-9F83-DF03AF116761}" uniqueName="10" name="Column10" queryTableFieldId="13" dataDxfId="45"/>
+    <tableColumn id="11" xr3:uid="{56D2129F-0933-4401-95C4-4829FF923A13}" uniqueName="11" name="Column11" queryTableFieldId="14" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1000,19 +1068,19 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C8257D7F-6FC7-48C3-94BB-5E01502C3467}" name="Table016__Page_92" displayName="Table016__Page_92" ref="A1:M11" tableType="queryTable" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{02D1957E-40E6-4536-885F-13BCFE4101C3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{2991BE4D-9578-46B8-BCEF-715B446423F5}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{ACCFCC68-FEF3-476F-9432-EF911E5D1A77}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{02D1957E-40E6-4536-885F-13BCFE4101C3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{2991BE4D-9578-46B8-BCEF-715B446423F5}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{ACCFCC68-FEF3-476F-9432-EF911E5D1A77}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="41"/>
     <tableColumn id="3" xr3:uid="{01736E20-EA76-45B7-87EA-536C6B1E165F}" uniqueName="3" name="Column3" queryTableFieldId="10"/>
     <tableColumn id="13" xr3:uid="{58900EE6-AE19-4A41-9876-6C4905A8347A}" uniqueName="13" name="Column13" queryTableFieldId="16"/>
-    <tableColumn id="5" xr3:uid="{E3A877E0-90AA-4B69-AD16-13D778CFC77C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{E3A877E0-90AA-4B69-AD16-13D778CFC77C}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="40"/>
     <tableColumn id="12" xr3:uid="{C3F104D0-15CF-4FB0-BEF1-080B2EC48D6D}" uniqueName="12" name="Column12" queryTableFieldId="15"/>
-    <tableColumn id="6" xr3:uid="{2B4B2FB0-1FC9-45C9-92D0-987D2AE90F09}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{EA6CCA08-9BDA-4C77-8A6F-554AEA83982B}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{1BF58AC6-F342-4F4C-80D2-0E40F741EE13}" uniqueName="8" name="Column8" queryTableFieldId="11" dataDxfId="27"/>
-    <tableColumn id="9" xr3:uid="{EDE40F09-A9EB-435F-A39A-22BCE532751A}" uniqueName="9" name="Column9" queryTableFieldId="12" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{44FBD4FB-4F8C-453A-BA41-FD5AAF52F2F5}" uniqueName="10" name="Column10" queryTableFieldId="13" dataDxfId="25"/>
-    <tableColumn id="11" xr3:uid="{44FBE715-568D-4715-83EB-E625AADB2D03}" uniqueName="11" name="Column11" queryTableFieldId="14" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{2B4B2FB0-1FC9-45C9-92D0-987D2AE90F09}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{EA6CCA08-9BDA-4C77-8A6F-554AEA83982B}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="38"/>
+    <tableColumn id="8" xr3:uid="{1BF58AC6-F342-4F4C-80D2-0E40F741EE13}" uniqueName="8" name="Column8" queryTableFieldId="11" dataDxfId="37"/>
+    <tableColumn id="9" xr3:uid="{EDE40F09-A9EB-435F-A39A-22BCE532751A}" uniqueName="9" name="Column9" queryTableFieldId="12" dataDxfId="36"/>
+    <tableColumn id="10" xr3:uid="{44FBD4FB-4F8C-453A-BA41-FD5AAF52F2F5}" uniqueName="10" name="Column10" queryTableFieldId="13" dataDxfId="35"/>
+    <tableColumn id="11" xr3:uid="{44FBE715-568D-4715-83EB-E625AADB2D03}" uniqueName="11" name="Column11" queryTableFieldId="14" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1021,9 +1089,9 @@
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{220B765F-DA51-4D95-AA58-E8416943B5C6}" name="Table017__Page_10" displayName="Table017__Page_10" ref="A1:I11" tableType="queryTable" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{90C90CD6-5F9E-4F28-81D5-B0222FD848F2}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{8A5B9A14-3872-4E3B-BC29-EB6B8C9FD996}" uniqueName="2" name="Technology" queryTableFieldId="2" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{204C75E9-84DB-49ED-B741-407B841543C3}" uniqueName="3" name="Zone" queryTableFieldId="3" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{90C90CD6-5F9E-4F28-81D5-B0222FD848F2}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{8A5B9A14-3872-4E3B-BC29-EB6B8C9FD996}" uniqueName="2" name="Technology" queryTableFieldId="2" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{204C75E9-84DB-49ED-B741-407B841543C3}" uniqueName="3" name="Zone" queryTableFieldId="3" dataDxfId="31"/>
     <tableColumn id="4" xr3:uid="{A488A660-5FBB-47B1-988D-4CBBF88DC623}" uniqueName="4" name="Bus" queryTableFieldId="4"/>
     <tableColumn id="7" xr3:uid="{3C751C34-5B6B-4703-9E6D-55D56287A813}" uniqueName="7" name="[MW]" queryTableFieldId="7"/>
     <tableColumn id="9" xr3:uid="{B8E6754C-F033-4C3A-8A1E-675E1D2716BA}" uniqueName="9" name="Column4" queryTableFieldId="14"/>
@@ -1038,16 +1106,16 @@
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FD7B0236-EBB8-4C35-B1F3-2548E9A3902C}" name="Table015__Page_8" displayName="Table015__Page_8" ref="A1:J6" tableType="queryTable" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{D120709C-B453-4249-9EA8-B1BB3B3A38D2}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{6AEAF6A5-29C8-4248-A153-84875D52D3F6}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{13501BF5-E17F-4544-BB83-6AD96E525790}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{B264AD4D-A011-465A-8ABB-DBEC93C50464}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{012ECDFC-F89D-443E-8C27-55F248C4C820}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{E79B387C-A0A8-46B2-981E-7A77BB823FC6}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{D120709C-B453-4249-9EA8-B1BB3B3A38D2}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{6AEAF6A5-29C8-4248-A153-84875D52D3F6}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{13501BF5-E17F-4544-BB83-6AD96E525790}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{B264AD4D-A011-465A-8ABB-DBEC93C50464}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{012ECDFC-F89D-443E-8C27-55F248C4C820}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{E79B387C-A0A8-46B2-981E-7A77BB823FC6}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="25"/>
     <tableColumn id="9" xr3:uid="{48DB4DAC-BDA3-47C9-92BC-2C3A44679F5D}" uniqueName="9" name="Column9" queryTableFieldId="10"/>
-    <tableColumn id="7" xr3:uid="{1FFFA2F9-ECD5-4AB6-B2AF-6AD10974455D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{F55DDDB2-769B-4C02-B497-6DA850D51883}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{0FE102E0-96C2-4E40-BA40-27763B43258E}" uniqueName="10" name="Column10" queryTableFieldId="11" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{1FFFA2F9-ECD5-4AB6-B2AF-6AD10974455D}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{F55DDDB2-769B-4C02-B497-6DA850D51883}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="23"/>
+    <tableColumn id="10" xr3:uid="{0FE102E0-96C2-4E40-BA40-27763B43258E}" uniqueName="10" name="Column10" queryTableFieldId="11" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1056,28 +1124,47 @@
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6D5A25C7-B3FD-4315-9AB6-C13858B8083C}" name="Table015__Page_88" displayName="Table015__Page_88" ref="A1:K25" tableType="queryTable" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{A3076C7B-B179-4467-AA62-6CB329A7BFFA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{8F5DDB80-92EF-40A9-9241-C853C92701C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{21212A2E-A7F6-48E3-8FFB-1930558EDD6F}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{BDD37EC8-9DCE-4814-BEDF-E92E3C2216CE}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{3499416A-AD34-45A6-82EE-D98B24A4D1F6}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{025CC4C5-D378-4A40-87CC-0889C41BE519}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{A3076C7B-B179-4467-AA62-6CB329A7BFFA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{8F5DDB80-92EF-40A9-9241-C853C92701C9}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{21212A2E-A7F6-48E3-8FFB-1930558EDD6F}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{BDD37EC8-9DCE-4814-BEDF-E92E3C2216CE}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{3499416A-AD34-45A6-82EE-D98B24A4D1F6}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{025CC4C5-D378-4A40-87CC-0889C41BE519}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="16"/>
     <tableColumn id="9" xr3:uid="{D3E91EC1-1B94-4B45-9D38-98FEE6B36876}" uniqueName="9" name="Column9" queryTableFieldId="10"/>
-    <tableColumn id="7" xr3:uid="{866F16E1-9BDC-4BAA-B80B-A640E0B956B8}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{39C22EC6-FE9B-484C-95AF-BEE19B6817EB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{1E462DD4-2B75-4360-8587-4195E771D301}" uniqueName="10" name="Column10" queryTableFieldId="11" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{EAD7ECDB-3FDC-4766-92FE-BD9869928CA4}" uniqueName="11" name="Column11" queryTableFieldId="12" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{866F16E1-9BDC-4BAA-B80B-A640E0B956B8}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{39C22EC6-FE9B-484C-95AF-BEE19B6817EB}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{1E462DD4-2B75-4360-8587-4195E771D301}" uniqueName="10" name="Column10" queryTableFieldId="11" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{EAD7ECDB-3FDC-4766-92FE-BD9869928CA4}" uniqueName="11" name="Column11" queryTableFieldId="12" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{0559ABF7-ACC9-4933-AECE-B39321DE4641}" name="Table015__Page_889" displayName="Table015__Page_889" ref="A1:K25" tableType="queryTable" headerRowCount="0" totalsRowShown="0">
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{CEFB1B2C-2689-4918-BBEB-E7EBDD9FCDAC}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{82CC6CB9-0095-42B7-AE71-B990261789EF}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{3C7112F2-69B7-4D27-B55C-3A0B779F1C5E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{5DC6C9B5-DDF3-4217-A97C-C88BBB308EB6}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{CFFE769F-6EC9-4728-A80F-D02AC996D953}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{D43D4E07-C80F-4B96-892A-26018939DA6F}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{27E9FB49-0E94-4356-B204-F40F15E883CC}" uniqueName="9" name="Column9" queryTableFieldId="10"/>
+    <tableColumn id="7" xr3:uid="{E9A7339B-3A0F-4D4D-AA7B-CB7D46B9816C}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{30D8CBB7-8C20-4C37-86F9-B55DCA1CE8C4}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{BF00F4BC-E59F-484B-A847-F47FFE8DDA44}" uniqueName="10" name="Column10" queryTableFieldId="11" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{9FB4782F-CD8B-4B5F-BF4F-3AAFB5B48356}" uniqueName="11" name="Column11" queryTableFieldId="12" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B98F3F0F-6FF3-4DF9-84FF-62DD8A59CE10}" name="Table018__Page_11" displayName="Table018__Page_11" ref="A1:H18" tableType="queryTable" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{E5811159-5BA9-4F6F-866C-A5B5FC14009E}" uniqueName="1" name="Load" queryTableFieldId="1"/>
     <tableColumn id="2" xr3:uid="{003C8E46-EE2F-46BC-ABEA-AAE7776BB7D5}" uniqueName="2" name="Bus" queryTableFieldId="2"/>
-    <tableColumn id="3" xr3:uid="{9E7C1477-C23B-44DD-B04E-225AAEF6399F}" uniqueName="3" name="Zone" queryTableFieldId="3" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{9E7C1477-C23B-44DD-B04E-225AAEF6399F}" uniqueName="3" name="Zone" queryTableFieldId="3" dataDxfId="11"/>
     <tableColumn id="6" xr3:uid="{F2077339-8203-40C7-81EB-C7E838CF0CFD}" uniqueName="6" name="[MW]" queryTableFieldId="6"/>
     <tableColumn id="8" xr3:uid="{42FF64AB-9053-4FFF-823A-A57A2D5F0737}" uniqueName="8" name="Column3" queryTableFieldId="10"/>
     <tableColumn id="7" xr3:uid="{37BF5EEB-BD2D-4F85-A4DB-FBCAE62042E9}" uniqueName="7" name="C_{d}^{LS} [$/MWh]" queryTableFieldId="7"/>
@@ -1088,12 +1175,12 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{F80E68BF-D9B2-4294-9556-931CE9087D56}" name="Table018__Page_117" displayName="Table018__Page_117" ref="A1:H18" tableType="queryTable" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{D225DC61-D286-4D1C-A363-65455C426366}" uniqueName="1" name="Load" queryTableFieldId="1"/>
     <tableColumn id="2" xr3:uid="{3C38AD07-246B-4A7E-A34D-B686DEF47E5F}" uniqueName="2" name="Bus" queryTableFieldId="2"/>
-    <tableColumn id="3" xr3:uid="{F52B33AC-C9D4-4B25-8526-26C1286B4B22}" uniqueName="3" name="Zone" queryTableFieldId="3" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{F52B33AC-C9D4-4B25-8526-26C1286B4B22}" uniqueName="3" name="Zone" queryTableFieldId="3" dataDxfId="10"/>
     <tableColumn id="6" xr3:uid="{BAAD1EF3-40F8-4EBF-B877-8E12A08ABEC1}" uniqueName="6" name="[MW]" queryTableFieldId="6"/>
     <tableColumn id="8" xr3:uid="{85EAD580-9079-449F-A971-F847AB8AC652}" uniqueName="8" name="Column3" queryTableFieldId="10"/>
     <tableColumn id="7" xr3:uid="{C1FD735E-0B29-4844-8CF8-F79BF56DA456}" uniqueName="7" name="C_{d}^{LS} [$/MWh]" queryTableFieldId="7"/>
@@ -2699,6 +2786,144 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22E32E64-9683-45C5-8A4E-FE0176A48B97}">
+  <dimension ref="A1:K22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" customWidth="1"/>
+    <col min="5" max="7" width="15" customWidth="1"/>
+    <col min="8" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>400</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1342000000000</v>
+      </c>
+      <c r="K2">
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B3" s="7"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="7"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B6" s="7"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J10" s="6"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B11" s="7"/>
+      <c r="J11" s="6"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J12" s="6"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B13" s="7"/>
+      <c r="J13" s="6"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B14" s="7"/>
+      <c r="J14" s="6"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J15" s="6"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J16" s="6"/>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J17" s="6"/>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B19" s="7"/>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B21" s="7"/>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B22" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{673DC82E-A05C-42A5-9C0F-ADF8689DC19F}">
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3189,7 +3414,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7645F89B-B6B6-480F-AB64-B9AA3BD498C6}">
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3680,7 +3905,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC66842A-8823-431E-9AA9-A5AC82E93231}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10981,7 +11206,7 @@
     <col min="4" max="4" width="14.7109375" customWidth="1"/>
     <col min="5" max="7" width="15" customWidth="1"/>
     <col min="8" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.85546875" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" customWidth="1"/>
     <col min="11" max="11" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Sync the line parameters used in the paper.
</commit_message>
<xml_diff>
--- a/data/rts_24_data.xlsx
+++ b/data/rts_24_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\repos\aro_tnep_sb_local\aro_tnep_sb\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ksorto\repos\aro_tnep_sb_local\aro_tnep_sb\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D400EA6-313C-4264-BF07-2AFDDF50079B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6052BE2B-E934-42DF-81EC-C327478C6123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6345" yWindow="3825" windowWidth="28800" windowHeight="15345" firstSheet="1" activeTab="2" xr2:uid="{61A108C2-359E-4CFD-B8CB-B26F47640E97}"/>
+    <workbookView xWindow="8910" yWindow="4365" windowWidth="28800" windowHeight="15345" firstSheet="1" activeTab="2" xr2:uid="{61A108C2-359E-4CFD-B8CB-B26F47640E97}"/>
   </bookViews>
   <sheets>
     <sheet name="TL" sheetId="1" r:id="rId1"/>
@@ -22,23 +22,26 @@
     <sheet name="RES" sheetId="4" r:id="rId7"/>
     <sheet name="ESS" sheetId="2" r:id="rId8"/>
     <sheet name="ESS_can" sheetId="15" r:id="rId9"/>
-    <sheet name="loads" sheetId="5" r:id="rId10"/>
-    <sheet name="loads_static" sheetId="14" r:id="rId11"/>
-    <sheet name="UB" sheetId="11" r:id="rId12"/>
+    <sheet name="ESS_none" sheetId="17" r:id="rId10"/>
+    <sheet name="loads" sheetId="5" r:id="rId11"/>
+    <sheet name="loads_static" sheetId="14" r:id="rId12"/>
+    <sheet name="UB" sheetId="11" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="ExternalData_1" localSheetId="4" hidden="1">CG!$A$1:$I$11</definedName>
     <definedName name="ExternalData_1" localSheetId="5" hidden="1">CG_static!$A$1:$I$11</definedName>
     <definedName name="ExternalData_1" localSheetId="7" hidden="1">ESS!$A$1:$I$6</definedName>
     <definedName name="ExternalData_1" localSheetId="8" hidden="1">ESS_can!$A$1:$I$25</definedName>
-    <definedName name="ExternalData_1" localSheetId="9" hidden="1">loads!$A$1:$F$18</definedName>
-    <definedName name="ExternalData_1" localSheetId="10" hidden="1">loads_static!$A$1:$F$18</definedName>
+    <definedName name="ExternalData_1" localSheetId="9" hidden="1">ESS_none!$A$1:$I$2</definedName>
+    <definedName name="ExternalData_1" localSheetId="10" hidden="1">loads!$A$1:$F$18</definedName>
+    <definedName name="ExternalData_1" localSheetId="11" hidden="1">loads_static!$A$1:$F$18</definedName>
     <definedName name="ExternalData_1" localSheetId="6" hidden="1">RES!$A$1:$G$11</definedName>
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">TL!$A$2:$F$56</definedName>
     <definedName name="ExternalData_1" localSheetId="2" hidden="1">TL_ESS!$A$2:$F$73</definedName>
     <definedName name="ExternalData_1" localSheetId="1" hidden="1">TL_static!$A$2:$F$73</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -138,7 +141,15 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="9" xr16:uid="{48047EF9-8182-45BF-9406-6828FCB3C1DB}" name="Query - Table013 (Page 7)" description="Connection to the 'Table013 (Page 7)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="9" xr16:uid="{759636A6-A5B3-42E9-A070-6AE42D6CAA27}" keepAlive="1" name="ModelConnection_ExternalData_18" description="Data Model" type="5" refreshedVersion="8" minRefreshableVersion="5" saveData="1">
+    <dbPr connection="Data Model Connection" command="Table015  Page 81" commandType="3"/>
+    <extLst>
+      <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
+        <x15:connection id="" model="1"/>
+      </ext>
+    </extLst>
+  </connection>
+  <connection id="10" xr16:uid="{48047EF9-8182-45BF-9406-6828FCB3C1DB}" name="Query - Table013 (Page 7)" description="Connection to the 'Table013 (Page 7)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="8c04846e-574b-49a9-b03c-b2747427d9dd">
@@ -151,7 +162,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="10" xr16:uid="{D25222F1-44AE-41FD-9C1A-34D8EC774F85}" name="Query - Table015 (Page 8)" description="Connection to the 'Table015 (Page 8)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="11" xr16:uid="{D25222F1-44AE-41FD-9C1A-34D8EC774F85}" name="Query - Table015 (Page 8)" description="Connection to the 'Table015 (Page 8)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="de4b364e-904d-453f-b309-9b29f4b6980b">
@@ -164,7 +175,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="11" xr16:uid="{9BE9130A-2930-4B7E-970E-BB06E9BF2541}" name="Query - Table015 (Page 8) (2)" description="Connection to the 'Table015 (Page 8) (2)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="12" xr16:uid="{9BE9130A-2930-4B7E-970E-BB06E9BF2541}" name="Query - Table015 (Page 8) (2)" description="Connection to the 'Table015 (Page 8) (2)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="bab8510e-8513-42ad-9cdf-1ac3ec4e9f1b">
@@ -177,7 +188,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="12" xr16:uid="{DB7B854D-31F1-4986-87EA-28D7E3F22A40}" name="Query - Table016 (Page 9)" description="Connection to the 'Table016 (Page 9)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="13" xr16:uid="{DB7B854D-31F1-4986-87EA-28D7E3F22A40}" name="Query - Table016 (Page 9)" description="Connection to the 'Table016 (Page 9)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="cac904aa-0e22-4628-a796-1353ff5a529d">
@@ -190,7 +201,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="13" xr16:uid="{59C9E23C-4A77-4FEB-8B7C-246516601062}" name="Query - Table017 (Page 10)" description="Connection to the 'Table017 (Page 10)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="14" xr16:uid="{59C9E23C-4A77-4FEB-8B7C-246516601062}" name="Query - Table017 (Page 10)" description="Connection to the 'Table017 (Page 10)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="d74bc432-1696-4381-8eaf-73d554f2c018">
@@ -203,7 +214,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="14" xr16:uid="{1721F4CF-7B60-4608-93AB-FAF0432B15AC}" name="Query - Table018 (Page 11)" description="Connection to the 'Table018 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="15" xr16:uid="{1721F4CF-7B60-4608-93AB-FAF0432B15AC}" name="Query - Table018 (Page 11)" description="Connection to the 'Table018 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="8c5efc9b-d372-436d-99c1-dde23be08897">
@@ -216,7 +227,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="15" xr16:uid="{A1A23163-EB73-4407-B25D-E8015E90F7B2}" name="Query - Table019 (Page 11)" description="Connection to the 'Table019 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="16" xr16:uid="{A1A23163-EB73-4407-B25D-E8015E90F7B2}" name="Query - Table019 (Page 11)" description="Connection to the 'Table019 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="4003258f-51d4-4a29-b633-006a99e36f39">
@@ -229,7 +240,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="16" xr16:uid="{36980317-2A15-439E-97F5-1B37DA855CA7}" name="Query - Table020 (Page 11)" description="Connection to the 'Table020 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
+  <connection id="17" xr16:uid="{36980317-2A15-439E-97F5-1B37DA855CA7}" name="Query - Table020 (Page 11)" description="Connection to the 'Table020 (Page 11)' query in the workbook." type="100" refreshedVersion="8" minRefreshableVersion="5">
     <extLst>
       <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
         <x15:connection id="1684410c-15f4-46ac-9515-2721589996c3">
@@ -242,7 +253,7 @@
       </ext>
     </extLst>
   </connection>
-  <connection id="17" xr16:uid="{91658BA7-C2B7-40CF-85C1-B529B7691349}" keepAlive="1" name="ThisWorkbookDataModel" description="Data Model" type="5" refreshedVersion="8" minRefreshableVersion="5" background="1">
+  <connection id="18" xr16:uid="{91658BA7-C2B7-40CF-85C1-B529B7691349}" keepAlive="1" name="ThisWorkbookDataModel" description="Data Model" type="5" refreshedVersion="8" minRefreshableVersion="5" background="1">
     <dbPr connection="Data Model Connection" command="Model" commandType="1"/>
     <olapPr sendLocale="1" rowDrillCount="1000"/>
     <extLst>
@@ -255,7 +266,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="91">
   <si>
     <t>Bus</t>
   </si>
@@ -629,7 +640,37 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="44">
+  <dxfs count="54">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -925,6 +966,34 @@
 </file>
 
 <file path=xl/queryTables/queryTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" headers="0" backgroundRefresh="0" connectionId="9" xr16:uid="{726C0C04-58E7-4812-9CDD-EC5B8C57EE32}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
+  <queryTableRefresh headersInLastRefresh="0" nextId="13" unboundColumnsRight="2">
+    <queryTableFields count="11">
+      <queryTableField id="1" name="Column1" tableColumnId="1"/>
+      <queryTableField id="2" name="Column2" tableColumnId="2"/>
+      <queryTableField id="3" name="Column3" tableColumnId="3"/>
+      <queryTableField id="4" name="Column4" tableColumnId="4"/>
+      <queryTableField id="5" name="Column5" tableColumnId="5"/>
+      <queryTableField id="6" name="Column6" tableColumnId="6"/>
+      <queryTableField id="10" dataBound="0" tableColumnId="9"/>
+      <queryTableField id="7" name="Column7" tableColumnId="7"/>
+      <queryTableField id="8" name="Column8" tableColumnId="8"/>
+      <queryTableField id="11" dataBound="0" tableColumnId="10"/>
+      <queryTableField id="12" dataBound="0" tableColumnId="11"/>
+    </queryTableFields>
+    <queryTableDeletedFields count="1">
+      <deletedField name="Column9"/>
+    </queryTableDeletedFields>
+  </queryTableRefresh>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{883FBD77-0823-4a55-B5E3-86C4891E6966}">
+      <x15:queryTable sourceDataName="Query - Table015 (Page 8) (2)"/>
+    </ext>
+  </extLst>
+</queryTable>
+</file>
+
+<file path=xl/queryTables/queryTable7.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" headers="0" backgroundRefresh="0" connectionId="5" xr16:uid="{77BA2001-87C6-4EE8-8DEC-2CF48E447D8D}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh headersInLastRefresh="0" nextId="11" unboundColumnsRight="2">
     <queryTableFields count="8">
@@ -950,7 +1019,7 @@
 </queryTable>
 </file>
 
-<file path=xl/queryTables/queryTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/queryTables/queryTable8.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" headers="0" backgroundRefresh="0" connectionId="7" xr16:uid="{BBD31A0C-45D3-4FA2-866B-846728885DB5}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh headersInLastRefresh="0" nextId="11" unboundColumnsRight="2">
     <queryTableFields count="8">
@@ -1073,6 +1142,25 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{C8BB39D3-4512-4DDB-95F6-7D8795FE3A4C}" name="Table015__Page_889" displayName="Table015__Page_889" ref="A1:K2" tableType="queryTable" headerRowCount="0" totalsRowShown="0">
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{8758AF1B-9325-4EEE-BF23-31109041FBEC}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{32BC9173-CB6C-4B71-BF76-97CAFAB985BA}" uniqueName="2" name="Column2" queryTableFieldId="2" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{EB5DD2E8-8241-4422-953D-C224EEA5BC4E}" uniqueName="3" name="Column3" queryTableFieldId="3" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{B8C12E19-4B7C-4052-907D-69ABA2057927}" uniqueName="4" name="Column4" queryTableFieldId="4" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{64109329-9A38-4A1B-A418-C01ED9A53E20}" uniqueName="5" name="Column5" queryTableFieldId="5" dataDxfId="49"/>
+    <tableColumn id="6" xr3:uid="{89DBAFA1-CBD6-4F8E-8191-E415A0C15661}" uniqueName="6" name="Column6" queryTableFieldId="6" dataDxfId="48"/>
+    <tableColumn id="9" xr3:uid="{1C37EBFC-A867-483C-BA31-3AA8B9972818}" uniqueName="9" name="Column9" queryTableFieldId="10"/>
+    <tableColumn id="7" xr3:uid="{F14C7E73-3656-4A3E-8B8D-723DED23A72E}" uniqueName="7" name="Column7" queryTableFieldId="7" dataDxfId="47"/>
+    <tableColumn id="8" xr3:uid="{D5A63ABF-F23C-4C3E-80E9-EA53F17EE71B}" uniqueName="8" name="Column8" queryTableFieldId="8" dataDxfId="46"/>
+    <tableColumn id="10" xr3:uid="{2114B860-62BD-4288-9143-03F90073E91C}" uniqueName="10" name="Column10" queryTableFieldId="11" dataDxfId="45"/>
+    <tableColumn id="11" xr3:uid="{814FD153-CF11-4B85-AEB8-4003B7ADD167}" uniqueName="11" name="Column11" queryTableFieldId="12" dataDxfId="44"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B98F3F0F-6FF3-4DF9-84FF-62DD8A59CE10}" name="Table018__Page_11" displayName="Table018__Page_11" ref="A1:H18" tableType="queryTable" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{E5811159-5BA9-4F6F-866C-A5B5FC14009E}" uniqueName="1" name="Load" queryTableFieldId="1"/>
@@ -1088,7 +1176,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{F80E68BF-D9B2-4294-9556-931CE9087D56}" name="Table018__Page_117" displayName="Table018__Page_117" ref="A1:H18" tableType="queryTable" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{D225DC61-D286-4D1C-A363-65455C426366}" uniqueName="1" name="Load" queryTableFieldId="1"/>
@@ -2699,6 +2787,99 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25FA0574-BAB2-4043-BC72-99D3C84A0EE5}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" customWidth="1"/>
+    <col min="5" max="7" width="15" customWidth="1"/>
+    <col min="8" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>400</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>134200000000</v>
+      </c>
+      <c r="K2">
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{673DC82E-A05C-42A5-9C0F-ADF8689DC19F}">
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3189,7 +3370,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7645F89B-B6B6-480F-AB64-B9AA3BD498C6}">
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3680,7 +3861,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC66842A-8823-431E-9AA9-A5AC82E93231}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6909,8 +7090,8 @@
         <v>1.4E-2</v>
       </c>
       <c r="E40">
-        <f>S40-50</f>
-        <v>100</v>
+        <f>S40</f>
+        <v>150</v>
       </c>
       <c r="F40">
         <f>H40</f>
@@ -6952,8 +7133,8 @@
         <v>1.4E-2</v>
       </c>
       <c r="E41">
-        <f t="shared" ref="E41:E87" si="1">S41-50</f>
-        <v>100</v>
+        <f t="shared" ref="E41:E87" si="1">S41</f>
+        <v>150</v>
       </c>
       <c r="F41">
         <f t="shared" ref="F41:F87" si="2">H41</f>
@@ -6996,7 +7177,7 @@
       </c>
       <c r="E42">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F42">
         <f t="shared" si="2"/>
@@ -7039,7 +7220,7 @@
       </c>
       <c r="E43">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F43">
         <f t="shared" si="2"/>
@@ -7082,7 +7263,7 @@
       </c>
       <c r="E44">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F44">
         <f t="shared" si="2"/>
@@ -7125,7 +7306,7 @@
       </c>
       <c r="E45">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F45">
         <f t="shared" si="2"/>
@@ -7168,7 +7349,7 @@
       </c>
       <c r="E46">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F46">
         <f t="shared" si="2"/>
@@ -7211,7 +7392,7 @@
       </c>
       <c r="E47">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F47">
         <f t="shared" si="2"/>
@@ -7254,7 +7435,7 @@
       </c>
       <c r="E48">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F48">
         <f t="shared" si="2"/>
@@ -7297,7 +7478,7 @@
       </c>
       <c r="E49">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F49">
         <f t="shared" si="2"/>
@@ -7340,7 +7521,7 @@
       </c>
       <c r="E50">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F50">
         <f t="shared" si="2"/>
@@ -7383,7 +7564,7 @@
       </c>
       <c r="E51">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F51">
         <f t="shared" si="2"/>
@@ -7426,7 +7607,7 @@
       </c>
       <c r="E52">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F52">
         <f t="shared" si="2"/>
@@ -7469,7 +7650,7 @@
       </c>
       <c r="E53">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F53">
         <f t="shared" si="2"/>
@@ -7512,7 +7693,7 @@
       </c>
       <c r="E54">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F54">
         <f t="shared" si="2"/>
@@ -7555,7 +7736,7 @@
       </c>
       <c r="E55">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F55">
         <f t="shared" si="2"/>
@@ -7598,7 +7779,7 @@
       </c>
       <c r="E56">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F56">
         <f t="shared" si="2"/>
@@ -7641,7 +7822,7 @@
       </c>
       <c r="E57">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F57">
         <f t="shared" si="2"/>
@@ -7684,7 +7865,7 @@
       </c>
       <c r="E58">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F58">
         <f t="shared" si="2"/>
@@ -7727,7 +7908,7 @@
       </c>
       <c r="E59">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F59">
         <f t="shared" si="2"/>
@@ -7770,7 +7951,7 @@
       </c>
       <c r="E60">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F60">
         <f t="shared" si="2"/>
@@ -7813,7 +7994,7 @@
       </c>
       <c r="E61">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F61">
         <f t="shared" si="2"/>
@@ -7856,7 +8037,7 @@
       </c>
       <c r="E62">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F62">
         <f t="shared" si="2"/>
@@ -7899,7 +8080,7 @@
       </c>
       <c r="E63">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F63">
         <f t="shared" si="2"/>
@@ -7942,7 +8123,7 @@
       </c>
       <c r="E64">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F64">
         <f t="shared" si="2"/>
@@ -7985,7 +8166,7 @@
       </c>
       <c r="E65">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F65">
         <f t="shared" si="2"/>
@@ -8028,7 +8209,7 @@
       </c>
       <c r="E66">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F66">
         <f t="shared" si="2"/>
@@ -8071,7 +8252,7 @@
       </c>
       <c r="E67">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F67">
         <f t="shared" si="2"/>
@@ -8114,7 +8295,7 @@
       </c>
       <c r="E68">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F68">
         <f t="shared" si="2"/>
@@ -8157,7 +8338,7 @@
       </c>
       <c r="E69">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F69">
         <f t="shared" si="2"/>
@@ -8200,7 +8381,7 @@
       </c>
       <c r="E70">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F70">
         <f t="shared" si="2"/>
@@ -8243,7 +8424,7 @@
       </c>
       <c r="E71">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F71">
         <f t="shared" si="2"/>
@@ -8286,7 +8467,7 @@
       </c>
       <c r="E72">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F72">
         <f t="shared" si="2"/>
@@ -8329,7 +8510,7 @@
       </c>
       <c r="E73">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F73">
         <f t="shared" si="2"/>
@@ -8372,7 +8553,7 @@
       </c>
       <c r="E74">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F74">
         <f t="shared" si="2"/>
@@ -8415,7 +8596,7 @@
       </c>
       <c r="E75">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F75">
         <f t="shared" si="2"/>
@@ -8458,7 +8639,7 @@
       </c>
       <c r="E76">
         <f t="shared" si="1"/>
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="F76">
         <f t="shared" si="2"/>
@@ -8501,7 +8682,7 @@
       </c>
       <c r="E77">
         <f t="shared" si="1"/>
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="F77">
         <f t="shared" si="2"/>
@@ -8544,7 +8725,7 @@
       </c>
       <c r="E78">
         <f t="shared" si="1"/>
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="F78">
         <f t="shared" si="2"/>
@@ -8587,7 +8768,7 @@
       </c>
       <c r="E79">
         <f t="shared" si="1"/>
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="F79">
         <f t="shared" si="2"/>
@@ -8630,7 +8811,7 @@
       </c>
       <c r="E80">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F80">
         <f t="shared" si="2"/>
@@ -8673,7 +8854,7 @@
       </c>
       <c r="E81">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F81">
         <f t="shared" si="2"/>
@@ -8716,7 +8897,7 @@
       </c>
       <c r="E82">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F82">
         <f t="shared" si="2"/>
@@ -8759,7 +8940,7 @@
       </c>
       <c r="E83">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F83">
         <f t="shared" si="2"/>
@@ -8802,7 +8983,7 @@
       </c>
       <c r="E84">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F84">
         <f t="shared" si="2"/>
@@ -8845,7 +9026,7 @@
       </c>
       <c r="E85">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F85">
         <f t="shared" si="2"/>
@@ -8888,7 +9069,7 @@
       </c>
       <c r="E86">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F86">
         <f t="shared" si="2"/>
@@ -8931,7 +9112,7 @@
       </c>
       <c r="E87">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F87">
         <f t="shared" si="2"/>

</xml_diff>